<commit_message>
xlstream-eval: extend issue-138 conditional fixture to 59 Excel-verified cases
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/issues/issue-138-bounded-conditional-aggregate.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/issues/issue-138-bounded-conditional-aggregate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream/crates/xlstream-eval/tests/fixtures/issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB238959-8E20-F547-BCC6-E0067F554B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89140679-576C-4046-B9A0-AFFA8E79617E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="91">
   <si>
     <t>num</t>
   </si>
@@ -256,6 +256,36 @@
   </si>
   <si>
     <t>COUNTIF whole-column &lt;&gt; numeric (blanks count as not-equal)</t>
+  </si>
+  <si>
+    <t>MINIFS bounded (sentinel C13 excluded)</t>
+  </si>
+  <si>
+    <t>MINIFS whole-column (negative sentinel included)</t>
+  </si>
+  <si>
+    <t>MAXIFS bounded (sentinel C12 excluded)</t>
+  </si>
+  <si>
+    <t>MAXIFS whole-column (sentinel included)</t>
+  </si>
+  <si>
+    <t>MINIFS bounded operator criteria (empty C cell ignored)</t>
+  </si>
+  <si>
+    <t>MAXIFS bounded operator criteria</t>
+  </si>
+  <si>
+    <t>MINIFS bounded no match returns 0</t>
+  </si>
+  <si>
+    <t>MAXIFS bounded no match returns 0</t>
+  </si>
+  <si>
+    <t>MINIFS mismatched range shapes VALUE</t>
+  </si>
+  <si>
+    <t>MAXIFS mismatched range shapes VALUE</t>
   </si>
   <si>
     <t>color</t>
@@ -616,13 +646,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="9" max="10" width="43.33203125" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -639,7 +666,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>10</v>
       </c>
@@ -655,15 +682,15 @@
       <c r="E2" t="s">
         <v>7</v>
       </c>
-      <c r="I2" t="s">
+      <c r="H2" t="s">
         <v>8</v>
       </c>
-      <c r="J2">
+      <c r="I2">
         <f>COUNTIF(A2:A11,50)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>20</v>
       </c>
@@ -676,15 +703,15 @@
       <c r="E3" t="s">
         <v>10</v>
       </c>
-      <c r="I3" t="s">
+      <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="J3">
+      <c r="I3">
         <f>COUNTIF(A:A,50)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>30</v>
       </c>
@@ -700,15 +727,15 @@
       <c r="E4" t="s">
         <v>13</v>
       </c>
-      <c r="I4" t="s">
+      <c r="H4" t="s">
         <v>14</v>
       </c>
-      <c r="J4">
+      <c r="I4">
         <f>COUNTIF(A2:A11,"&gt;50")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>40</v>
       </c>
@@ -721,15 +748,15 @@
       <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="I5" t="s">
+      <c r="H5" t="s">
         <v>17</v>
       </c>
-      <c r="J5">
+      <c r="I5">
         <f>COUNTIF(A2:A11,"=50")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>50</v>
       </c>
@@ -739,15 +766,15 @@
       <c r="E6" t="s">
         <v>18</v>
       </c>
-      <c r="I6" t="s">
+      <c r="H6" t="s">
         <v>19</v>
       </c>
-      <c r="J6">
+      <c r="I6">
         <f>COUNTIF(A2:A11,"&lt;&gt;50")</f>
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>60</v>
       </c>
@@ -763,15 +790,15 @@
       <c r="E7" t="s">
         <v>22</v>
       </c>
-      <c r="I7" t="s">
+      <c r="H7" t="s">
         <v>23</v>
       </c>
-      <c r="J7">
+      <c r="I7">
         <f>COUNTIF(B2:B11,"east")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>70</v>
       </c>
@@ -784,15 +811,15 @@
       <c r="E8" t="s">
         <v>25</v>
       </c>
-      <c r="I8" t="s">
+      <c r="H8" t="s">
         <v>26</v>
       </c>
-      <c r="J8">
+      <c r="I8">
         <f>COUNTIF(B:B,"east")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>80</v>
       </c>
@@ -805,15 +832,15 @@
       <c r="E9" t="s">
         <v>7</v>
       </c>
-      <c r="I9" t="s">
+      <c r="H9" t="s">
         <v>27</v>
       </c>
-      <c r="J9">
+      <c r="I9">
         <f>COUNTIF(E2:E11,"ap*")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>-10</v>
       </c>
@@ -829,15 +856,15 @@
       <c r="E10" t="s">
         <v>29</v>
       </c>
-      <c r="I10" t="s">
+      <c r="H10" t="s">
         <v>30</v>
       </c>
-      <c r="J10">
+      <c r="I10">
         <f>COUNTIF(E2:E11,"?pple")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>5.5</v>
       </c>
@@ -850,15 +877,15 @@
       <c r="E11" t="s">
         <v>31</v>
       </c>
-      <c r="I11" t="s">
+      <c r="H11" t="s">
         <v>32</v>
       </c>
-      <c r="J11">
+      <c r="I11">
         <f>COUNTIF(E2:E11,"&gt;banana")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>9999</v>
       </c>
@@ -874,15 +901,15 @@
       <c r="E12" t="s">
         <v>7</v>
       </c>
-      <c r="I12" t="s">
+      <c r="H12" t="s">
         <v>34</v>
       </c>
-      <c r="J12">
+      <c r="I12">
         <f>COUNTIF(D2:D11,"")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>50</v>
       </c>
@@ -890,353 +917,443 @@
         <v>5</v>
       </c>
       <c r="C13">
-        <v>88888</v>
+        <v>-7777</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
       </c>
-      <c r="I13" t="s">
+      <c r="H13" t="s">
         <v>35</v>
       </c>
-      <c r="J13">
+      <c r="I13">
         <f>COUNTIF(D2:D11,"&lt;&gt;")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I14" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H14" t="s">
         <v>36</v>
       </c>
-      <c r="J14">
+      <c r="I14">
         <f>COUNTIF(A2:A11,"&lt;0")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I15" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H15" t="s">
         <v>37</v>
       </c>
-      <c r="J15">
+      <c r="I15">
         <f>COUNTIF(A2:A11,777)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G16" t="s">
         <v>38</v>
       </c>
-      <c r="I16" t="s">
+      <c r="H16" t="s">
         <v>39</v>
       </c>
-      <c r="J16">
+      <c r="I16">
         <f>COUNTIF(A2:A11,G16)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I17" t="s">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H17" t="s">
         <v>40</v>
       </c>
-      <c r="J17">
+      <c r="I17">
         <f>SUMIF(A2:A11,"&gt;50")</f>
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I18" t="s">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H18" t="s">
         <v>41</v>
       </c>
-      <c r="J18">
+      <c r="I18">
         <f>SUMIF(A:A,"&gt;50")</f>
         <v>10209</v>
       </c>
     </row>
-    <row r="19" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I19" t="s">
+    <row r="19" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H19" t="s">
         <v>42</v>
       </c>
-      <c r="J19">
+      <c r="I19">
         <f>SUMIF(B2:B11,"east",C2:C11)</f>
         <v>1200</v>
       </c>
     </row>
-    <row r="20" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I20" t="s">
+    <row r="20" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H20" t="s">
         <v>43</v>
       </c>
-      <c r="J20">
+      <c r="I20">
         <f>SUMIF(B:B,"east",C:C)</f>
-        <v>190087</v>
-      </c>
-    </row>
-    <row r="21" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I21" t="s">
+        <v>93422</v>
+      </c>
+    </row>
+    <row r="21" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H21" t="s">
         <v>44</v>
       </c>
-      <c r="J21">
+      <c r="I21">
         <f>SUMIF(E2:E11,"ap*",C2:C11)</f>
         <v>1800</v>
       </c>
     </row>
-    <row r="22" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I22" t="s">
+    <row r="22" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H22" t="s">
         <v>45</v>
       </c>
-      <c r="J22">
+      <c r="I22">
         <f>SUMIF(A2:A11,"=50")</f>
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I23" t="s">
+    <row r="23" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H23" t="s">
         <v>46</v>
       </c>
-      <c r="J23">
+      <c r="I23">
         <f>SUMIF(A2:A11,777)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I24" t="s">
+    <row r="24" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H24" t="s">
         <v>47</v>
       </c>
-      <c r="J24">
+      <c r="I24">
         <f>SUMIF(D2:D11,"",C2:C11)</f>
         <v>3100</v>
       </c>
     </row>
-    <row r="25" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I25" t="s">
+    <row r="25" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H25" t="s">
         <v>48</v>
       </c>
-      <c r="J25">
+      <c r="I25">
         <f>AVERAGEIF(A2:A11,"&gt;0")</f>
         <v>40.611111111111114</v>
       </c>
     </row>
-    <row r="26" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I26" t="s">
+    <row r="26" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H26" t="s">
         <v>49</v>
       </c>
-      <c r="J26">
+      <c r="I26">
         <f>AVERAGEIF(B2:B11,"east",C2:C11)</f>
         <v>400</v>
       </c>
     </row>
-    <row r="27" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I27" t="s">
+    <row r="27" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H27" t="s">
         <v>50</v>
       </c>
-      <c r="J27" t="e">
+      <c r="I27" t="e">
         <f>AVERAGEIF(A2:A11,777)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="28" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I28" t="s">
+    <row r="28" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H28" t="s">
         <v>51</v>
       </c>
-      <c r="J28">
+      <c r="I28">
         <f>AVERAGEIF(A2:A11,"&lt;0")</f>
         <v>-10</v>
       </c>
     </row>
-    <row r="29" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I29" t="s">
+    <row r="29" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H29" t="s">
         <v>52</v>
       </c>
-      <c r="J29">
+      <c r="I29">
         <f>COUNTIFS(B2:B11,"east",A2:A11,"&gt;30")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I30" t="s">
+    <row r="30" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H30" t="s">
         <v>53</v>
       </c>
-      <c r="J30">
+      <c r="I30">
         <f>COUNTIFS(B:B,"east",A:A,"&gt;30")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I31" t="s">
+    <row r="31" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H31" t="s">
         <v>54</v>
       </c>
-      <c r="J31">
+      <c r="I31">
         <f>COUNTIFS(B2:B11,"east")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I32" t="s">
+    <row r="32" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H32" t="s">
         <v>55</v>
       </c>
-      <c r="J32" t="e">
+      <c r="I32" t="e">
         <f>COUNTIFS(B2:B11,"east",A2:A12,"&gt;30")</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="33" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I33" t="s">
+    <row r="33" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H33" t="s">
         <v>56</v>
       </c>
-      <c r="J33">
+      <c r="I33">
         <f>COUNTIFS(E2:E11,"ap*",A2:A11,"&lt;100")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I34" t="s">
+    <row r="34" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H34" t="s">
         <v>57</v>
       </c>
-      <c r="J34">
+      <c r="I34">
         <f>SUMIFS(C2:C11,B2:B11,"east",A2:A11,"&gt;30")</f>
         <v>800</v>
       </c>
     </row>
-    <row r="35" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I35" t="s">
+    <row r="35" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H35" t="s">
         <v>58</v>
       </c>
-      <c r="J35">
+      <c r="I35">
         <f>SUMIFS(C:C,B:B,"east",A:A,"&gt;30")</f>
-        <v>189687</v>
-      </c>
-    </row>
-    <row r="36" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I36" t="s">
+        <v>93022</v>
+      </c>
+    </row>
+    <row r="36" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H36" t="s">
         <v>59</v>
       </c>
-      <c r="J36" t="e">
+      <c r="I36" t="e">
         <f>SUMIFS(C2:C11,B2:B11,"east",A2:A10,"&gt;30")</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="37" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I37" t="s">
+    <row r="37" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H37" t="s">
         <v>60</v>
       </c>
-      <c r="J37">
+      <c r="I37">
         <f>SUMIFS(C2:C11,E2:E11,"ap*")</f>
         <v>1800</v>
       </c>
     </row>
-    <row r="38" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I38" t="s">
+    <row r="38" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H38" t="s">
         <v>61</v>
       </c>
-      <c r="J38">
+      <c r="I38">
         <f>AVERAGEIFS(C2:C11,B2:B11,"east",A2:A11,"&gt;30")</f>
         <v>800</v>
       </c>
     </row>
-    <row r="39" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I39" t="s">
+    <row r="39" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H39" t="s">
         <v>62</v>
       </c>
-      <c r="J39" t="e">
+      <c r="I39" t="e">
         <f>AVERAGEIFS(C2:C11,B2:B11,"nomatch")</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="40" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I40" t="s">
+    <row r="40" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H40" t="s">
         <v>63</v>
       </c>
-      <c r="J40" t="e">
+      <c r="I40" t="e">
         <f>AVERAGEIFS(C2:C11,B2:B11,"east",A2:A12,"&gt;30")</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="41" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I41" t="s">
+    <row r="41" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H41" t="s">
         <v>64</v>
       </c>
-      <c r="J41">
+      <c r="I41">
         <f>COUNTIF(Ref!A2:A11,"red")</f>
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I42" t="s">
+    <row r="42" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H42" t="s">
         <v>65</v>
       </c>
-      <c r="J42">
+      <c r="I42">
         <f>COUNTIF(Ref!A:A,"red")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I43" t="s">
+    <row r="43" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H43" t="s">
         <v>66</v>
       </c>
-      <c r="J43">
+      <c r="I43">
         <f>SUMIF(Ref!A2:A11,"red",Ref!B2:B11)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I44" t="s">
+    <row r="44" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H44" t="s">
         <v>67</v>
       </c>
-      <c r="J44">
+      <c r="I44">
         <f>SUMIF(Ref!A:A,"red",Ref!B:B)</f>
         <v>3016</v>
       </c>
     </row>
-    <row r="45" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I45" t="s">
+    <row r="45" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H45" t="s">
         <v>68</v>
       </c>
-      <c r="J45">
+      <c r="I45">
         <f>SUMIFS(Ref!B2:B11,Ref!A2:A11,"red")</f>
         <v>16</v>
       </c>
     </row>
-    <row r="46" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I46" t="s">
+    <row r="46" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H46" t="s">
         <v>69</v>
       </c>
-      <c r="J46">
+      <c r="I46">
         <f>AVERAGEIF(Ref!A2:A11,"red",Ref!B2:B11)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I47" t="s">
+    <row r="47" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H47" t="s">
         <v>70</v>
       </c>
-      <c r="J47">
+      <c r="I47">
         <f>COUNTIFS(Ref!A2:A11,"red",Ref!B2:B11,"&gt;4")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I48" t="s">
+    <row r="48" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H48" t="s">
         <v>71</v>
       </c>
-      <c r="J48">
+      <c r="I48">
         <f>COUNTIF(D:D,"")</f>
         <v>1048570</v>
       </c>
     </row>
-    <row r="49" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I49" t="s">
+    <row r="49" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H49" t="s">
         <v>72</v>
       </c>
-      <c r="J49">
+      <c r="I49">
         <f>COUNTIF(D:D,"&lt;&gt;")</f>
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I50" t="s">
+    <row r="50" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H50" t="s">
         <v>73</v>
       </c>
-      <c r="J50">
+      <c r="I50">
         <f>COUNTIF(A:A,"&lt;&gt;50")</f>
         <v>1048574</v>
+      </c>
+    </row>
+    <row r="51" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H51" t="s">
+        <v>74</v>
+      </c>
+      <c r="I51">
+        <f>_xlfn.MINIFS(C2:C11,B2:B11,"east")</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H52" t="s">
+        <v>75</v>
+      </c>
+      <c r="I52">
+        <f>_xlfn.MINIFS(C:C,B:B,"east")</f>
+        <v>-7777</v>
+      </c>
+    </row>
+    <row r="53" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H53" t="s">
+        <v>76</v>
+      </c>
+      <c r="I53">
+        <f>_xlfn.MAXIFS(C2:C11,B2:B11,"east")</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="54" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H54" t="s">
+        <v>77</v>
+      </c>
+      <c r="I54">
+        <f>_xlfn.MAXIFS(C:C,B:B,"east")</f>
+        <v>99999</v>
+      </c>
+    </row>
+    <row r="55" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H55" t="s">
+        <v>78</v>
+      </c>
+      <c r="I55">
+        <f>_xlfn.MINIFS(C2:C11,A2:A11,"&gt;30")</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="56" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H56" t="s">
+        <v>79</v>
+      </c>
+      <c r="I56">
+        <f>_xlfn.MAXIFS(C2:C11,A2:A11,"&gt;30")</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="57" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H57" t="s">
+        <v>80</v>
+      </c>
+      <c r="I57">
+        <f>_xlfn.MINIFS(C2:C11,B2:B11,"nomatch")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H58" t="s">
+        <v>81</v>
+      </c>
+      <c r="I58">
+        <f>_xlfn.MAXIFS(C2:C11,B2:B11,"nomatch")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H59" t="s">
+        <v>82</v>
+      </c>
+      <c r="I59" t="e">
+        <f>_xlfn.MINIFS(C2:C11,B2:B11,"east",A2:A12,"&gt;0")</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="60" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H60" t="s">
+        <v>83</v>
+      </c>
+      <c r="I60" t="e">
+        <f>_xlfn.MAXIFS(C2:C11,B2:B11,"east",A2:A12,"&gt;0")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -1251,15 +1368,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1267,7 +1384,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1275,7 +1392,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1283,7 +1400,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -1291,7 +1408,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1299,7 +1416,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -1307,7 +1424,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -1315,7 +1432,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -1323,7 +1440,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -1331,7 +1448,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1339,7 +1456,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B12">
         <v>1000</v>
@@ -1347,7 +1464,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="B13">
         <v>2000</v>

</xml_diff>